<commit_message>
Etapa 1: reporte Bitcoin con Excel
</commit_message>
<xml_diff>
--- a/output/reporte.xlsx
+++ b/output/reporte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>Precio USD</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Fecha consulta</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -435,7 +440,42 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80075</v>
+        <v>81458</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2376.5</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Litecoin</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>56.51</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:59</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Etapa 2: Excel, CSV, HTML, PDF y zona horaria Argentina
</commit_message>
<xml_diff>
--- a/output/reporte.xlsx
+++ b/output/reporte.xlsx
@@ -440,11 +440,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81458</v>
+        <v>60260</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-05 21:59</t>
+          <t>2026-06-24 13:40</t>
         </is>
       </c>
     </row>
@@ -455,11 +455,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2376.5</v>
+        <v>1623.7</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-05 21:59</t>
+          <t>2026-06-24 13:40</t>
         </is>
       </c>
     </row>
@@ -470,11 +470,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56.51</v>
+        <v>40.84</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-05 21:59</t>
+          <t>2026-06-24 13:40</t>
         </is>
       </c>
     </row>

</xml_diff>